<commit_message>
[refactor] UI 구조 개선
[UIManager 구조 개선]
Inspector에 프리팹을 하나씩 등록 -> Addressables 일괄 로드 방식으로 변경.
GameManager에서 데이터 로드 → UI 프리팹 로드 → DataInitialized 발행 순서로 초기화 흐름 제어.
BindState가 일치하는 UI는 전부 스폰, Auto 여부로 즉시 표시/대기 분리

[StageClear / StageFailed]
게임 상태 변경 관련 팝업은 이벤트 구독 방식으로 변경.
GamePlayUI에서 직접 OpenUI 호출 제거 → OnStageClear / OnStageFailed 구독해서 스스로 열림.

[레이어 위반 수정]
StationController → UIManager 직접 참조 제거.
OnStationInteractionChanged 이벤트에 StationController 참조를 실어 발행,
UIManager가 구독해서 StationUpgrade 열고 닫는 책임 인수.
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/UI.xlsx
+++ b/JsonConverter/ExcelFiles/UI.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="14568" windowHeight="8400"/>
+    <workbookView windowWidth="13128" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="40">
   <si>
     <t>아이디</t>
   </si>
@@ -41,7 +41,7 @@
     <t>게임 상태 바인딩</t>
   </si>
   <si>
-    <t>상태 진입시 자동 스폰 여부</t>
+    <t>자동으로 열림 여부</t>
   </si>
   <si>
     <t>string</t>
@@ -68,82 +68,70 @@
     <t>BindState</t>
   </si>
   <si>
-    <t>AutoSpawn</t>
-  </si>
-  <si>
-    <t>UI_Popup_01</t>
-  </si>
-  <si>
-    <t>OpenedStage</t>
+    <t>Auto</t>
+  </si>
+  <si>
+    <t>UI_Popup_03</t>
+  </si>
+  <si>
+    <t>StageClear</t>
   </si>
   <si>
     <t>Popup</t>
   </si>
   <si>
+    <t>GamePlay</t>
+  </si>
+  <si>
+    <t>false</t>
+  </si>
+  <si>
+    <t>UI_Popup_04</t>
+  </si>
+  <si>
+    <t>StageFailed</t>
+  </si>
+  <si>
+    <t>UI_Popup_05</t>
+  </si>
+  <si>
+    <t>StageStart</t>
+  </si>
+  <si>
+    <t>UI_Popup_06</t>
+  </si>
+  <si>
+    <t>PlanetInfo</t>
+  </si>
+  <si>
+    <t>UI_Popup_07</t>
+  </si>
+  <si>
+    <t>StationUpgrade</t>
+  </si>
+  <si>
+    <t>UI_Panel_01</t>
+  </si>
+  <si>
+    <t>MainMenu</t>
+  </si>
+  <si>
+    <t>Main</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>UI_Panel_02</t>
+  </si>
+  <si>
+    <t>UI_Panel_03</t>
+  </si>
+  <si>
+    <t>GameLobby</t>
+  </si>
+  <si>
     <t>Lobby</t>
-  </si>
-  <si>
-    <t>false</t>
-  </si>
-  <si>
-    <t>UI_Popup_02</t>
-  </si>
-  <si>
-    <t>ClosedStage</t>
-  </si>
-  <si>
-    <t>UI_Popup_03</t>
-  </si>
-  <si>
-    <t>StageClear</t>
-  </si>
-  <si>
-    <t>GamePlay</t>
-  </si>
-  <si>
-    <t>UI_Popup_04</t>
-  </si>
-  <si>
-    <t>StageFailed</t>
-  </si>
-  <si>
-    <t>UI_Popup_05</t>
-  </si>
-  <si>
-    <t>StageStart</t>
-  </si>
-  <si>
-    <t>UI_Popup_06</t>
-  </si>
-  <si>
-    <t>PlanetInfo</t>
-  </si>
-  <si>
-    <t>UI_Popup_07</t>
-  </si>
-  <si>
-    <t>StationUpgrade</t>
-  </si>
-  <si>
-    <t>UI_Panel_01</t>
-  </si>
-  <si>
-    <t>MainMenu</t>
-  </si>
-  <si>
-    <t>Main</t>
-  </si>
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>UI_Panel_02</t>
-  </si>
-  <si>
-    <t>UI_Panel_03</t>
-  </si>
-  <si>
-    <t>GameLobby</t>
   </si>
   <si>
     <t>UI_Panel_04</t>
@@ -1357,19 +1345,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G25"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="6"/>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="15.5555555555556" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="13.6666666666667" customWidth="1"/>
     <col min="4" max="4" width="16.5555555555556" customWidth="1"/>
-    <col min="5" max="5" width="24.2222222222222" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="32.2222222222222" customWidth="1"/>
+    <col min="5" max="5" width="20.2222222222222" style="1" customWidth="1"/>
+    <col min="6" max="6" width="32.2222222222222" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1385,10 +1372,9 @@
       <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3"/>
-      <c r="G1" s="5"/>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="F1" s="5"/>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -1404,10 +1390,9 @@
       <c r="E2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="3"/>
-      <c r="G2" s="5"/>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="F2" s="5"/>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
@@ -1423,14 +1408,13 @@
       <c r="E3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="5"/>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="F3" s="5"/>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C4" s="3" t="s">
@@ -1442,14 +1426,12 @@
       <c r="E4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="5"/>
-    </row>
-    <row r="5" spans="1:7">
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C5" s="3" t="s">
@@ -1461,10 +1443,8 @@
       <c r="E5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="5"/>
-    </row>
-    <row r="6" spans="1:7">
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
@@ -1475,254 +1455,200 @@
         <v>16</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="2"/>
-    </row>
-    <row r="7" spans="1:7">
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" spans="1:7">
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="2"/>
-    </row>
-    <row r="9" spans="1:7">
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="D9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" s="2"/>
-    </row>
-    <row r="10" spans="1:7">
+        <v>28</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F10" s="2"/>
-    </row>
-    <row r="11" spans="1:7">
+    </row>
+    <row r="11" customFormat="1" spans="1:6">
       <c r="A11" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>33</v>
-      </c>
       <c r="E11" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F11" s="2"/>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="C12" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>23</v>
-      </c>
       <c r="E12" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="F12" s="2"/>
-    </row>
-    <row r="13" customFormat="1" spans="1:7">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>17</v>
+      <c r="C13" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>38</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="F15" s="2"/>
-    </row>
-    <row r="16" spans="1:7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="8"/>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="2"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="8"/>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
       <c r="E16" s="8"/>
-      <c r="F16" s="2"/>
-    </row>
-    <row r="17" spans="1:6">
+    </row>
+    <row r="17" spans="1:5">
       <c r="A17" s="2"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
       <c r="E17" s="8"/>
-      <c r="F17" s="2"/>
-    </row>
-    <row r="18" spans="1:6">
+    </row>
+    <row r="18" spans="1:5">
       <c r="A18" s="2"/>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="8"/>
-      <c r="F18" s="2"/>
-    </row>
-    <row r="19" spans="1:6">
+    </row>
+    <row r="19" spans="1:5">
       <c r="A19" s="2"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
       <c r="E19" s="8"/>
-      <c r="F19" s="2"/>
-    </row>
-    <row r="20" spans="1:6">
+    </row>
+    <row r="20" spans="1:5">
       <c r="A20" s="2"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
       <c r="E20" s="8"/>
-      <c r="F20" s="2"/>
-    </row>
-    <row r="21" spans="1:6">
+    </row>
+    <row r="21" spans="1:5">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="8"/>
-      <c r="F21" s="2"/>
-    </row>
-    <row r="22" spans="1:6">
+    </row>
+    <row r="22" spans="1:5">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="8"/>
-      <c r="F22" s="2"/>
-    </row>
-    <row r="23" spans="1:6">
+    </row>
+    <row r="23" spans="1:5">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="8"/>
-      <c r="F23" s="2"/>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="2"/>
-    </row>
-    <row r="25" spans="1:6">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
[Add] 랭크(Scoreboard) 시스템 설계
[추가]
- 스테이지 클리어시의 점수와 날짜를 보관하고, 이를 점수값으로 정렬한 순위표 팝업 추가
- 데이터의 갯수만큼 Item을 동적 생성하도록 설계, 자동 정렬을 위해 Vertical Layout Group, Content Size Fitter 사용
- 원안은 Score를 Key로 SortedDictionary 사용 예정이었으나, 스테이지 Id 기반으로 클리어 여부 및 기록을 조회해야 하므로 스테이지 Id를 Key로 사용하는 Dictionary로 변경
- 표시 시점에 최대 5개만 List.Sort()로 정렬 (데이터가 많지 않아 비용을 무시함)
- LobbyUI에서 현재 선택된 스테이지 Id를 직접 캐싱하여 스테이지별 독립 점수판 보장
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/UI.xlsx
+++ b/JsonConverter/ExcelFiles/UI.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="13776" windowHeight="8400"/>
+    <workbookView windowWidth="16524" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="50">
   <si>
     <t>아이디</t>
   </si>
@@ -131,6 +131,15 @@
     <t>StationMarket</t>
   </si>
   <si>
+    <t>UI_Popup_09</t>
+  </si>
+  <si>
+    <t>Scoreboard</t>
+  </si>
+  <si>
+    <t>Lobby</t>
+  </si>
+  <si>
     <t>UI_Panel_01</t>
   </si>
   <si>
@@ -147,9 +156,6 @@
   </si>
   <si>
     <t>GameLobby</t>
-  </si>
-  <si>
-    <t>Lobby</t>
   </si>
   <si>
     <t>UI_Panel_04</t>
@@ -1378,7 +1384,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="15.5555555555556" customWidth="1"/>
@@ -1584,16 +1590,16 @@
         <v>34</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="11" t="s">
         <v>36</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -1601,50 +1607,50 @@
         <v>37</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="3" t="s">
+      <c r="C14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" customFormat="1" spans="1:6">
-      <c r="A14" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="12" t="s">
+      <c r="E14" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
+    </row>
+    <row r="15" customFormat="1" spans="1:6">
       <c r="A15" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="12" t="s">
         <v>42</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1654,39 +1660,49 @@
       <c r="B16" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>44</v>
+      <c r="C16" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E17" s="11" t="s">
+      <c r="D18" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="2"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="11"/>
+      <c r="E18" s="11" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="2"/>
@@ -1711,9 +1727,9 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
       <c r="E22" s="11"/>
     </row>
     <row r="23" spans="1:5">
@@ -1744,6 +1760,13 @@
       <c r="D26" s="2"/>
       <c r="E26" s="11"/>
     </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="11"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
[refactor] UIManagerExtension 분리 / CurrencyUI 구조 개선
[추가]
- 게임 흐름에 따라 동작하는 UI들을 확장 메서드 방식으로 분리
=> UIManager는 UI들의 공통 로직만 남기고 상세한 동작은 Extension에서 처리
[수정]
- CurrencyUI를 데이터에 등록
- CurrencyUI를 UIBase를 상속하도록 변경
=> 이벤트 구독/해제 방식을 통일
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/UI.xlsx
+++ b/JsonConverter/ExcelFiles/UI.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="23040" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="62">
   <si>
     <t>아이디</t>
   </si>
@@ -168,6 +168,12 @@
   </si>
   <si>
     <t>Achievement</t>
+  </si>
+  <si>
+    <t>UI_Panel_06</t>
+  </si>
+  <si>
+    <t>Currency</t>
   </si>
   <si>
     <t>UI_Loading_01</t>
@@ -1414,7 +1420,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="15.5555555555556" customWidth="1"/>
@@ -1724,44 +1730,44 @@
       <c r="B18" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>48</v>
-      </c>
+      <c r="C18" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" s="3"/>
       <c r="E18" s="11" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>36</v>
+      <c r="D19" s="12" t="s">
+        <v>50</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C20" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="D20" s="12"/>
+      <c r="C20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="E20" s="11" t="s">
         <v>17</v>
       </c>
@@ -1773,8 +1779,8 @@
       <c r="B21" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>49</v>
+      <c r="C21" s="12" t="s">
+        <v>51</v>
       </c>
       <c r="D21" s="12"/>
       <c r="E21" s="11" t="s">
@@ -1788,8 +1794,8 @@
       <c r="B22" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>16</v>
+      <c r="C22" s="3" t="s">
+        <v>51</v>
       </c>
       <c r="D22" s="12"/>
       <c r="E22" s="11" t="s">
@@ -1812,11 +1818,19 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="11"/>
+      <c r="A24" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="12"/>
+      <c r="E24" s="11" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="2"/>
@@ -1846,6 +1860,13 @@
       <c r="D28" s="2"/>
       <c r="E28" s="11"/>
     </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="11"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
[Add] Setting, Option 추가
[추가]
- MainMenu - Option 버튼 활성화 및 클릭시 팝업 구현
=> 배경음, 효과음 볼륨 Slider 및 텍스트 연동
- Looby/GamePlay - Setting 토글 버튼 구현
=> BGM ON/OFF 기능, GamePlay -> Lobby, Lobby -> MainMenu 버튼 구현
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/UI.xlsx
+++ b/JsonConverter/ExcelFiles/UI.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8400"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="66">
   <si>
     <t>아이디</t>
   </si>
@@ -140,6 +140,12 @@
     <t>Lobby</t>
   </si>
   <si>
+    <t>UI_Popup_10</t>
+  </si>
+  <si>
+    <t>Option</t>
+  </si>
+  <si>
     <t>UI_Panel_01</t>
   </si>
   <si>
@@ -174,6 +180,12 @@
   </si>
   <si>
     <t>Currency</t>
+  </si>
+  <si>
+    <t>UI_Panel_07</t>
+  </si>
+  <si>
+    <t>Setting</t>
   </si>
   <si>
     <t>UI_Loading_01</t>
@@ -1420,7 +1432,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="15.5555555555556" customWidth="1"/>
@@ -1643,67 +1655,67 @@
         <v>37</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="11" t="s">
-        <v>39</v>
+      <c r="E13" s="4" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="D14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="3" t="s">
+      <c r="C15" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="15" customFormat="1" spans="1:6">
-      <c r="A15" s="2" t="s">
+      <c r="E15" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
+    </row>
+    <row r="16" customFormat="1" spans="1:6">
       <c r="A16" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="12" t="s">
         <v>44</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>36</v>
       </c>
       <c r="E16" s="11" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1714,7 +1726,7 @@
         <v>46</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>36</v>
@@ -1731,11 +1743,13 @@
         <v>48</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D18" s="3"/>
+        <v>40</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>36</v>
+      </c>
       <c r="E18" s="11" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1745,59 +1759,59 @@
       <c r="B19" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="D19" s="12" t="s">
-        <v>50</v>
-      </c>
+      <c r="C19" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="3"/>
       <c r="E19" s="11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>36</v>
-      </c>
+      <c r="C20" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D20" s="3"/>
       <c r="E20" s="11" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="C21" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="D21" s="12"/>
+      <c r="D21" s="12" t="s">
+        <v>54</v>
+      </c>
       <c r="E21" s="11" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D22" s="12"/>
+      <c r="C22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="E22" s="11" t="s">
         <v>17</v>
       </c>
@@ -1809,8 +1823,8 @@
       <c r="B23" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>16</v>
+      <c r="C23" s="12" t="s">
+        <v>55</v>
       </c>
       <c r="D23" s="12"/>
       <c r="E23" s="11" t="s">
@@ -1824,8 +1838,8 @@
       <c r="B24" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>16</v>
+      <c r="C24" s="3" t="s">
+        <v>55</v>
       </c>
       <c r="D24" s="12"/>
       <c r="E24" s="11" t="s">
@@ -1833,18 +1847,34 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="11"/>
+      <c r="A25" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D25" s="12"/>
+      <c r="E25" s="11" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="11"/>
+      <c r="A26" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D26" s="12"/>
+      <c r="E26" s="11" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="2"/>
@@ -1867,6 +1897,20 @@
       <c r="D29" s="2"/>
       <c r="E29" s="11"/>
     </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="11"/>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="2"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="11"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>